<commit_message>
Beginning error bus integration, defining project layers. Need to look into proper scaffolding separation for app and core modules.
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/orders/A.L. George/A.L. George_Collegetown_20251114.xlsx
+++ b/WorkBot/refactor-experimental/data/orders/A.L. George/A.L. George_Collegetown_20251114.xlsx
@@ -454,20 +454,14 @@
           <t>Guayaki Yerba Mate - Enlighten Mint</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>26.00</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>26.00</t>
-        </is>
+      <c r="C2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" t="n">
+        <v>26</v>
+      </c>
+      <c r="E2" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="3">
@@ -481,20 +475,14 @@
           <t>Essentia Water</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>16.50</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>33.00</t>
-        </is>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -508,20 +496,14 @@
           <t>Evian 1L</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>23.00</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>46.00</t>
-        </is>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>23</v>
+      </c>
+      <c r="E4" t="n">
+        <v>46</v>
       </c>
     </row>
     <row r="5">
@@ -535,20 +517,14 @@
           <t>Fiji Water 500ml</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>18.50</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>37.00</t>
-        </is>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E5" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="6">
@@ -562,20 +538,14 @@
           <t>Ithaca Soda - Root Beer</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>23.95</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>23.95</t>
-        </is>
+      <c r="C6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" t="n">
+        <v>23.95</v>
+      </c>
+      <c r="E6" t="n">
+        <v>23.95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Some file restructuring, realization of over-engineering; enjoyment nonetheless.
</commit_message>
<xml_diff>
--- a/WorkBot/refactor-experimental/data/orders/A.L. George/A.L. George_Collegetown_20251114.xlsx
+++ b/WorkBot/refactor-experimental/data/orders/A.L. George/A.L. George_Collegetown_20251114.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,105 +446,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>77220</t>
+          <t>75155</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Guayaki Yerba Mate - Enlighten Mint</t>
+          <t>Essentia Water</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>16.5</v>
       </c>
       <c r="E2" t="n">
-        <v>26</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>75155</t>
+          <t>74602</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Essentia Water</t>
+          <t>Evian 1L</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>16.5</v>
+        <v>23</v>
       </c>
       <c r="E3" t="n">
-        <v>33</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>74602</t>
+          <t>75101</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Evian 1L</t>
+          <t>Fiji Water 500ml</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>23</v>
+        <v>18.5</v>
       </c>
       <c r="E4" t="n">
-        <v>46</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>75101</t>
+          <t>77801</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fiji Water 500ml</t>
+          <t>Ithaca Soda - Root Beer</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>18.5</v>
+        <v>23.95</v>
       </c>
       <c r="E5" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>77801</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Ithaca Soda - Root Beer</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="n">
-        <v>23.95</v>
-      </c>
-      <c r="E6" t="n">
         <v>23.95</v>
       </c>
     </row>

</xml_diff>